<commit_message>
code added for Italy
</commit_message>
<xml_diff>
--- a/Data/Hires/testDataUS.xlsx
+++ b/Data/Hires/testDataUS.xlsx
@@ -507,52 +507,46 @@
     <t>Test_14</t>
   </si>
   <si>
-    <t xml:space="preserve">Test failed for 'Madelynn Yost' Employee:{10652380}Error: [2mexpect([22m[31mreceived[39m[2m).[22mtoEqual[2m([22m[32mexpected[39m[2m) // deep equality[22m
-Expected: [32m"USA Pay Group"[39m
-Received: [31m"[7mPlease select a [27mUSA Pay Group"[39m</t>
-  </si>
-  <si>
-    <t>Madelynn</t>
-  </si>
-  <si>
-    <t>Yost</t>
-  </si>
-  <si>
-    <t>Auto 65006340</t>
+    <t>10652410</t>
+  </si>
+  <si>
+    <t>Karli</t>
+  </si>
+  <si>
+    <t>Kris</t>
+  </si>
+  <si>
+    <t>Auto 39710683</t>
   </si>
   <si>
     <t>Test_15</t>
   </si>
   <si>
-    <t xml:space="preserve">Test failed for 'Katelynn Rohan' Employee:{10652385}Error: [2mexpect([22m[31mreceived[39m[2m).[22mtoEqual[2m([22m[32mexpected[39m[2m) // deep equality[22m
-Expected: [32m"USA Pay Group"[39m
-Received: [31m"[7mPlease select a [27mUSA Pay Group"[39m</t>
-  </si>
-  <si>
-    <t>Katelynn</t>
-  </si>
-  <si>
-    <t>Rohan</t>
-  </si>
-  <si>
-    <t>Auto 79007249</t>
+    <t>10652407</t>
+  </si>
+  <si>
+    <t>Philip</t>
+  </si>
+  <si>
+    <t>Crooks</t>
+  </si>
+  <si>
+    <t>Auto 6318502</t>
   </si>
   <si>
     <t>Test_16</t>
   </si>
   <si>
-    <t xml:space="preserve">Test failed for 'Glen Wolf' Employee:{10652395}Error: [2mexpect([22m[31mreceived[39m[2m).[22mtoEqual[2m([22m[32mexpected[39m[2m) // deep equality[22m
-Expected: [32m"USA Pay Group"[39m
-Received: [31m"[7mPlease select a [27mUSA Pay Group"[39m</t>
+    <t>10652405</t>
   </si>
   <si>
     <t>108 Recruitment (Pepog Bizyse (10240565))</t>
   </si>
   <si>
-    <t>Glen</t>
-  </si>
-  <si>
-    <t>Wolf</t>
+    <t>Kyler</t>
+  </si>
+  <si>
+    <t>Schaefer</t>
   </si>
   <si>
     <t>No</t>
@@ -674,7 +668,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
+        <fgColor rgb="FF00FF00"/>
       </patternFill>
     </fill>
     <fill>
@@ -772,7 +766,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -902,6 +896,9 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1557,7 +1554,7 @@
       </c>
       <c r="AS2" s="28">
         <f t="array" ref="AS2:AS17">_xlfn.RANDARRAY(16,1,123456789,999999999,FALSE)</f>
-        <v>382384988.3993381</v>
+        <v>460815640.7913228</v>
       </c>
       <c r="AT2" s="22" t="s">
         <v>83</v>
@@ -1727,7 +1724,7 @@
         <v>82</v>
       </c>
       <c r="AS3" s="28">
-        <v>520899656.7887391</v>
+        <v>472982800.79699147</v>
       </c>
       <c r="AT3" s="39" t="s">
         <v>83</v>
@@ -1900,7 +1897,7 @@
         <v>82</v>
       </c>
       <c r="AS4" s="28">
-        <v>557812545.4056697</v>
+        <v>318166387.0177647</v>
       </c>
       <c r="AT4" s="22" t="s">
         <v>83</v>
@@ -2073,7 +2070,7 @@
         <v>82</v>
       </c>
       <c r="AS5" s="28">
-        <v>989456017.6990048</v>
+        <v>467531187.97844076</v>
       </c>
       <c r="AT5" s="22" t="s">
         <v>83</v>
@@ -2246,7 +2243,7 @@
         <v>82</v>
       </c>
       <c r="AS6" s="28">
-        <v>785876381.062165</v>
+        <v>517755556.7426585</v>
       </c>
       <c r="AT6" s="22" t="s">
         <v>83</v>
@@ -2419,7 +2416,7 @@
         <v>82</v>
       </c>
       <c r="AS7" s="28">
-        <v>804058163.7429827</v>
+        <v>555811152.5144323</v>
       </c>
       <c r="AT7" s="22" t="s">
         <v>83</v>
@@ -2589,7 +2586,7 @@
         <v>82</v>
       </c>
       <c r="AS8" s="28">
-        <v>632508201.5898451</v>
+        <v>825511269.0782044</v>
       </c>
       <c r="AT8" s="39" t="s">
         <v>83</v>
@@ -2762,7 +2759,7 @@
         <v>82</v>
       </c>
       <c r="AS9" s="28">
-        <v>784364524.2209965</v>
+        <v>747492505.429115</v>
       </c>
       <c r="AT9" s="22" t="s">
         <v>83</v>
@@ -2935,7 +2932,7 @@
         <v>82</v>
       </c>
       <c r="AS10" s="28">
-        <v>690276280.6384156</v>
+        <v>927618183.0344183</v>
       </c>
       <c r="AT10" s="22" t="s">
         <v>83</v>
@@ -3105,7 +3102,7 @@
         <v>82</v>
       </c>
       <c r="AS11" s="28">
-        <v>501541083.3148836</v>
+        <v>687838782.7348971</v>
       </c>
       <c r="AT11" s="39" t="s">
         <v>83</v>
@@ -3278,7 +3275,7 @@
         <v>82</v>
       </c>
       <c r="AS12" s="28">
-        <v>660781998.1587614</v>
+        <v>830591566.4173034</v>
       </c>
       <c r="AT12" s="22" t="s">
         <v>83</v>
@@ -3451,7 +3448,7 @@
         <v>82</v>
       </c>
       <c r="AS13" s="28">
-        <v>369519756.158321</v>
+        <v>892760956.1489455</v>
       </c>
       <c r="AT13" s="22" t="s">
         <v>83</v>
@@ -3491,7 +3488,7 @@
       <c r="A14" t="s">
         <v>153</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="52" t="s">
         <v>154</v>
       </c>
       <c r="C14" s="7" t="s">
@@ -3621,7 +3618,7 @@
         <v>82</v>
       </c>
       <c r="AS14" s="28">
-        <v>584522102.083316</v>
+        <v>788948433.5635042</v>
       </c>
       <c r="AT14" s="39" t="s">
         <v>83</v>
@@ -3665,7 +3662,7 @@
         <v>163</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>121</v>
+        <v>55</v>
       </c>
       <c r="D15" s="50" t="s">
         <v>155</v>
@@ -3794,7 +3791,7 @@
         <v>82</v>
       </c>
       <c r="AS15" s="28">
-        <v>407198291.49721277</v>
+        <v>584250515.7309579</v>
       </c>
       <c r="AT15" s="22" t="s">
         <v>83</v>
@@ -3838,7 +3835,7 @@
         <v>168</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>121</v>
+        <v>55</v>
       </c>
       <c r="D16" s="50" t="s">
         <v>155</v>
@@ -3967,7 +3964,7 @@
         <v>82</v>
       </c>
       <c r="AS16" s="28">
-        <v>419288037.28788507</v>
+        <v>227977938.30577552</v>
       </c>
       <c r="AT16" s="22" t="s">
         <v>83</v>
@@ -4007,11 +4004,11 @@
       <c r="A17" t="s">
         <v>172</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="52" t="s">
         <v>173</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>121</v>
+        <v>55</v>
       </c>
       <c r="D17" s="50" t="s">
         <v>174</v>
@@ -4137,12 +4134,12 @@
         <v>82</v>
       </c>
       <c r="AS17" s="28">
-        <v>696712179.0472647</v>
+        <v>153729041.11979425</v>
       </c>
       <c r="AT17" s="39" t="s">
         <v>83</v>
       </c>
-      <c r="AU17" s="52" t="s">
+      <c r="AU17" s="53" t="s">
         <v>184</v>
       </c>
       <c r="AV17" s="26" t="s">
@@ -4174,7 +4171,7 @@
       </c>
     </row>
     <row r="18" ht="14.5" customHeight="1" spans="45:45" x14ac:dyDescent="0.25">
-      <c r="AS18" s="53"/>
+      <c r="AS18" s="54"/>
     </row>
   </sheetData>
   <dataValidations count="24">

</xml_diff>